<commit_message>
add Exercise 4A to w2_workshop
</commit_message>
<xml_diff>
--- a/Merawi_Ex3A_tables.xlsx
+++ b/Merawi_Ex3A_tables.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yearuptemp-my.sharepoint.com/personal/hmerawi_my_yearupunited_org/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yearuptemp-my.sharepoint.com/personal/hmerawi_my_yearupunited_org/Documents/Desktop/Documents/DataAnalytics/week-02/W2_Workshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="8_{FBD3E8D6-415D-48EC-AE57-B171D7FDBADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F61187C-C9AC-4849-885D-F98FAD9D36F6}"/>
+  <xr:revisionPtr revIDLastSave="136" documentId="8_{FBD3E8D6-415D-48EC-AE57-B171D7FDBADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19AF8E09-76A0-42C3-94B4-FCF2E4BE31C6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{61A552F9-B89F-4862-B4D3-1872C3DD18F3}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Customer" sheetId="1" r:id="rId1"/>
     <sheet name="Dog" sheetId="2" r:id="rId2"/>
     <sheet name="Walk" sheetId="3" r:id="rId3"/>
-    <sheet name="walker" sheetId="4" r:id="rId4"/>
+    <sheet name="walkers" sheetId="4" r:id="rId4"/>
     <sheet name="Payment" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -40,10 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
-  <si>
-    <t>owner_id</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="44">
   <si>
     <t>first_name</t>
   </si>
@@ -63,9 +60,6 @@
     <t>dog_id</t>
   </si>
   <si>
-    <t>owener_id</t>
-  </si>
-  <si>
     <t>name</t>
   </si>
   <si>
@@ -75,9 +69,6 @@
     <t>age</t>
   </si>
   <si>
-    <t>medical_note</t>
-  </si>
-  <si>
     <t>walk_id</t>
   </si>
   <si>
@@ -115,16 +106,90 @@
   </si>
   <si>
     <t>method</t>
+  </si>
+  <si>
+    <t>Kennedy</t>
+  </si>
+  <si>
+    <t>571-456-2589</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>john.kennedy@email.com</t>
+  </si>
+  <si>
+    <t>123 silent tree pl</t>
+  </si>
+  <si>
+    <t>emergency_contact</t>
+  </si>
+  <si>
+    <t>John Kennedy 571-456-2589</t>
+  </si>
+  <si>
+    <t>Maribella</t>
+  </si>
+  <si>
+    <t>Bob</t>
+  </si>
+  <si>
+    <t>maribella.b@gmail.com</t>
+  </si>
+  <si>
+    <t>789-564-1236</t>
+  </si>
+  <si>
+    <t>Lead Walker</t>
+  </si>
+  <si>
+    <t>Rocky</t>
+  </si>
+  <si>
+    <t>Boxer</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>medical_notes</t>
+  </si>
+  <si>
+    <t>No Poultry</t>
+  </si>
+  <si>
+    <t>Scheduled</t>
+  </si>
+  <si>
+    <t>Morning park walk</t>
+  </si>
+  <si>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>Completed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -159,15 +224,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -504,27 +574,124 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34EB69A1-E88D-430D-B5ED-DE3C7CD8BE0E}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.88671875" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" customWidth="1"/>
+    <col min="6" max="6" width="17.21875" customWidth="1"/>
+    <col min="7" max="7" width="24.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{80007CFE-7AA1-4126-AF2B-D5BEC9DD5ABF}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D8F7EC1-8240-4AD0-8D03-2CE351F7FD01}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
       <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="C2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
-        <v>5</v>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -532,32 +699,61 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D8F7EC1-8240-4AD0-8D03-2CE351F7FD01}">
-  <dimension ref="A1:F1"/>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC62E9AA-D907-47E3-B131-AD4AD7797DDA}">
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="6" max="6" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" customWidth="1"/>
+    <col min="5" max="5" width="14.77734375" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" t="s">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4">
+        <v>46143</v>
+      </c>
+      <c r="E2" s="5">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="F2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -565,112 +761,129 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC62E9AA-D907-47E3-B131-AD4AD7797DDA}">
-  <dimension ref="A1:G1"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8674A196-F17C-4D16-B8DF-92BD8B9415D8}">
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="14.109375" customWidth="1"/>
-    <col min="5" max="5" width="14.77734375" customWidth="1"/>
+    <col min="1" max="2" width="9.44140625" customWidth="1"/>
+    <col min="3" max="3" width="9.5546875" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" customWidth="1"/>
+    <col min="5" max="5" width="15.5546875" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>16</v>
       </c>
-      <c r="G1" t="s">
-        <v>17</v>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" s="4">
+        <v>46037</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{A38E07BB-5B92-4F22-82C1-D46D88E9E7BB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8674A196-F17C-4D16-B8DF-92BD8B9415D8}">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="9.44140625" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" customWidth="1"/>
-    <col min="4" max="4" width="9.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3B6A13D-5188-4194-9184-A0DBFFA9D6FF}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.5546875" customWidth="1"/>
     <col min="2" max="2" width="10.88671875" customWidth="1"/>
     <col min="5" max="5" width="12.109375" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" t="s">
-        <v>24</v>
-      </c>
       <c r="G1" t="s">
-        <v>16</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>30</v>
+      </c>
+      <c r="E2" s="4">
+        <v>46144</v>
+      </c>
+      <c r="F2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>